<commit_message>
Aggregate output to one row per athlete (summed score)
Change the primary output from one row per performance to one row per
athlete, identified by the composite key (NAME, ID, COLLEGE). A single
athlete may have multiple event entries in the input; their World Athletics
points are now summed into a single total SCORE.

- models.py: add AthleteAggregate and AGGREGATE_COLUMNS (NAME, ID, COLLEGE,
  GENDER, SCORE)
- scorer.py: add aggregate_by_athlete() grouping by composite key,
  case/space-insensitive, sorted by descending total
- writer.py: Results sheet is now per-athlete; add a Details sheet with the
  per-performance breakdown grouped under each athlete
- main.py: aggregate after scoring; add --no-details; log distinct athletes
- examples: add multi-event athletes to demonstrate summation
- tests: add aggregation coverage (22 tests pass)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0119jtmkdE2GaNSVKUhWNHvR
</commit_message>
<xml_diff>
--- a/examples/example_input.xlsx
+++ b/examples/example_input.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1196,17 +1196,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bad Event</t>
+          <t>Aarav Sharma</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>X001</t>
+          <t>M001</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Unknown College</t>
+          <t>Fergusson College</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Tug of War</t>
+          <t>Long Jump</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1226,42 +1226,190 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>5.00</t>
+          <t>7.10</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>Aarav Sharma</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Fergusson College</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>200m</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>21.90</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Priya Menon</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>W001</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Fergusson College</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>200m</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>24.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Priya Menon</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>W001</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Fergusson College</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Long Jump</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>DISTANCE</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>5.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Bad Event</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>X001</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Unknown College</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Tug of War</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>DISTANCE</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>5.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>Bad Result</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>X002</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Unknown College</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>100m</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>TIME</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>not-a-time</t>
         </is>

</xml_diff>

<commit_message>
cli+examples: add --mapping option and bib-based example files
- main.py: add optional -m/--mapping to enrich output via a BIB->identity
  file; load it through the loader, apply after aggregation, and rank
  colleges from the enriched data; clear error on an invalid mapping
- examples/generate_example_input.py: emit a bib-keyed main file
  (example_input.xlsx/.csv) plus an optional mapping file
  (example_mapping.xlsx/.csv). The sample deliberately leaves one bib
  unmapped and one college blank to exercise those paths
- regenerate example_output.xlsx (enriched, with College Ranking)

Verified: with mapping -> enriched Results + College Ranking; without
mapping -> bib-only Results and no College Ranking sheet; empty bib rejected.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0119jtmkdE2GaNSVKUhWNHvR
</commit_message>
<xml_diff>
--- a/examples/example_input.xlsx
+++ b/examples/example_input.xlsx
@@ -413,41 +413,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>NAME</t>
+          <t>BIB NUMBER</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>GENDER</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>COLLEGE</t>
+          <t>EVENT NAME</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>GENDER</t>
+          <t>PERFORMANCE TYPE</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
-        <is>
-          <t>EVENT NAME</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>PERFORMANCE TYPE</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
         <is>
           <t>RESULT</t>
         </is>
@@ -456,35 +446,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Aarav Sharma</t>
+          <t>101</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>M001</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fergusson College</t>
+          <t>100m</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
-        <is>
-          <t>100m</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
         <is>
           <t>10.87</t>
         </is>
@@ -493,35 +473,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Rahul Verma</t>
+          <t>102</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>M002</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>St. Xavier's</t>
+          <t>200m</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
-        <is>
-          <t>200m</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
         <is>
           <t>21.44</t>
         </is>
@@ -530,35 +500,25 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Karan Patel</t>
+          <t>103</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>M003</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Loyola College</t>
+          <t>400m</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
-        <is>
-          <t>400m</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
         <is>
           <t>48.90</t>
         </is>
@@ -567,35 +527,25 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Vikram Singh</t>
+          <t>104</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>M004</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fergusson College</t>
+          <t>800m</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
-        <is>
-          <t>800m</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
         <is>
           <t>1:52.30</t>
         </is>
@@ -604,35 +554,25 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Arjun Nair</t>
+          <t>105</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>M005</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Christ University</t>
+          <t>1500m</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
-        <is>
-          <t>1500m</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
         <is>
           <t>3:55.10</t>
         </is>
@@ -641,35 +581,25 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rohan Das</t>
+          <t>106</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>M006</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>St. Xavier's</t>
+          <t>110m Hurdles</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
-        <is>
-          <t>110m Hurdles</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
         <is>
           <t>14.55</t>
         </is>
@@ -678,35 +608,25 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Aditya Rao</t>
+          <t>107</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>M007</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Loyola College</t>
+          <t>Long Jump</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>DISTANCE</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
-        <is>
-          <t>Long Jump</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>DISTANCE</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
         <is>
           <t>7.35</t>
         </is>
@@ -715,35 +635,25 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sameer Khan</t>
+          <t>108</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>M008</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Christ University</t>
+          <t>Shot Put</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>DISTANCE</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
-        <is>
-          <t>Shot Put</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>DISTANCE</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
         <is>
           <t>16.20</t>
         </is>
@@ -752,35 +662,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Nikhil Reddy</t>
+          <t>109</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>M009</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fergusson College</t>
+          <t>Javelin Throw</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>DISTANCE</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
-        <is>
-          <t>Javelin Throw</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>DISTANCE</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
         <is>
           <t>68.40</t>
         </is>
@@ -789,35 +689,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Gupta</t>
+          <t>110</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>M010</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>St. Xavier's</t>
+          <t>High Jump</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>DISTANCE</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
-        <is>
-          <t>High Jump</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>DISTANCE</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
         <is>
           <t>2.10</t>
         </is>
@@ -826,35 +716,25 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Priya Menon</t>
+          <t>201</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>W001</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fergusson College</t>
+          <t>100m</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
-        <is>
-          <t>100m</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
         <is>
           <t>11.90</t>
         </is>
@@ -863,35 +743,25 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sneha Iyer</t>
+          <t>202</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>W002</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>St. Xavier's</t>
+          <t>200m</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
-        <is>
-          <t>200m</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
         <is>
           <t>24.30</t>
         </is>
@@ -900,35 +770,25 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ananya Bose</t>
+          <t>203</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>W003</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Loyola College</t>
+          <t>400m</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
-        <is>
-          <t>400m</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
         <is>
           <t>54.20</t>
         </is>
@@ -937,35 +797,25 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Divya Pillai</t>
+          <t>204</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>W004</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Christ University</t>
+          <t>800m</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
-        <is>
-          <t>800m</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
         <is>
           <t>2:05.31</t>
         </is>
@@ -974,35 +824,25 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Meera Joshi</t>
+          <t>205</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>W005</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fergusson College</t>
+          <t>100m Hurdles</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
-        <is>
-          <t>100m Hurdles</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
         <is>
           <t>13.85</t>
         </is>
@@ -1011,35 +851,25 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Kavya Nair</t>
+          <t>206</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>W006</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>St. Xavier's</t>
+          <t>Long Jump</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>DISTANCE</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
-        <is>
-          <t>Long Jump</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>DISTANCE</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
         <is>
           <t>6.35</t>
         </is>
@@ -1048,35 +878,25 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ritika Shah</t>
+          <t>207</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>W007</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Loyola College</t>
+          <t>Shot Put</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>DISTANCE</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
-        <is>
-          <t>Shot Put</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>DISTANCE</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
         <is>
           <t>14.10</t>
         </is>
@@ -1085,35 +905,25 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Pooja Desai</t>
+          <t>208</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>W008</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Christ University</t>
+          <t>Javelin Throw</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>DISTANCE</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
-        <is>
-          <t>Javelin Throw</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>DISTANCE</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
         <is>
           <t>52.35</t>
         </is>
@@ -1122,35 +932,25 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Isha Kapoor</t>
+          <t>209</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>W009</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Fergusson College</t>
+          <t>High Jump</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>DISTANCE</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
-        <is>
-          <t>High Jump</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>DISTANCE</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
         <is>
           <t>1.82</t>
         </is>
@@ -1159,35 +959,25 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Tanvi Rao</t>
+          <t>210</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>W010</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>St. Xavier's</t>
+          <t>1500m</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
-        <is>
-          <t>1500m</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
         <is>
           <t>4:15.60</t>
         </is>
@@ -1196,35 +986,25 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Aarav Sharma</t>
+          <t>101</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>M001</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Fergusson College</t>
+          <t>Long Jump</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>DISTANCE</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
-        <is>
-          <t>Long Jump</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>DISTANCE</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
         <is>
           <t>7.10</t>
         </is>
@@ -1233,35 +1013,25 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aarav Sharma</t>
+          <t>101</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>M001</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Fergusson College</t>
+          <t>200m</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
-        <is>
-          <t>200m</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
         <is>
           <t>21.90</t>
         </is>
@@ -1270,35 +1040,25 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Priya Menon</t>
+          <t>201</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>W001</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Fergusson College</t>
+          <t>200m</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
-        <is>
-          <t>200m</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
         <is>
           <t>24.10</t>
         </is>
@@ -1307,35 +1067,25 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Priya Menon</t>
+          <t>201</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>W001</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Fergusson College</t>
+          <t>Long Jump</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>DISTANCE</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
-        <is>
-          <t>Long Jump</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>DISTANCE</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
         <is>
           <t>5.95</t>
         </is>
@@ -1344,35 +1094,25 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Bad Event</t>
+          <t>901</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>X001</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Unknown College</t>
+          <t>Tug of War</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>DISTANCE</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
-        <is>
-          <t>Tug of War</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>DISTANCE</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
         <is>
           <t>5.00</t>
         </is>
@@ -1381,37 +1121,50 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Bad Result</t>
+          <t>902</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>X002</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Unknown College</t>
+          <t>100m</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
+          <t>not-a-time</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
           <t>100m</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>not-a-time</t>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>10.50</t>
         </is>
       </c>
     </row>

</xml_diff>